<commit_message>
Actualizo productos, precios y stock
</commit_message>
<xml_diff>
--- a/catalogo_productos_banco.xlsx
+++ b/catalogo_productos_banco.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="355">
   <si>
     <t xml:space="preserve">CATÁLOGO BANCO DE SUPLEMENTOS — No editar este archivo con otras herramientas</t>
   </si>
@@ -124,60 +124,63 @@
     <t xml:space="preserve">true</t>
   </si>
   <si>
+    <t xml:space="preserve">Creatina Monohidrato 300g magali</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Star Nutrition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">supplements</t>
+  </si>
+  <si>
+    <t xml:space="preserve">creatines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">creatina-star-300g.webp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">light</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Más Vendido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Creatina monohidrato micronizada Star Nutrition 300g. Clínicamente probada para aumentar la fuerza, la potencia y la masa muscular magra. El suplemento más estudiado en nutrición deportiva.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">300g en polvo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sin sabor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuerza y Potencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disolvé 1 porción (5g) en 200–300 ml de agua o jugo. Tomá una vez al día, preferentemente post-entrenamiento o con una comida. Etapa de carga opcional: 4 porciones diarias durante los primeros 5–7 días para saturar reservas más rápido.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aumentá la fuerza máxima, la potencia explosiva y la masa muscular magra. La creatina es el suplemento más estudiado de la nutrición deportiva, con evidencia sólida para musculación, CrossFit, sprint y actividades de alta intensidad.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">creatina-star-300g-tabla.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">whey-gentech-500g-chocolate, combo-proteina-creatina-gentech</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://wa.me/5491124602875?text=Hola%2C%20me%20interesa%20la%20Creatina%20Monohidrato%20300g%20Star%20Nutrition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">creatina-granger-300g</t>
+  </si>
+  <si>
     <t xml:space="preserve">Creatina Monohidrato 300g</t>
   </si>
   <si>
-    <t xml:space="preserve">Star Nutrition</t>
-  </si>
-  <si>
-    <t xml:space="preserve">supplements</t>
-  </si>
-  <si>
-    <t xml:space="preserve">creatines</t>
-  </si>
-  <si>
-    <t xml:space="preserve">creatina-star-300g.webp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">light</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Más Vendido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Creatina monohidrato micronizada Star Nutrition 300g. Clínicamente probada para aumentar la fuerza, la potencia y la masa muscular magra. El suplemento más estudiado en nutrición deportiva.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">300g en polvo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sin sabor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuerza y Potencia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Disolvé 1 porción (5g) en 200–300 ml de agua o jugo. Tomá una vez al día, preferentemente post-entrenamiento o con una comida. Etapa de carga opcional: 4 porciones diarias durante los primeros 5–7 días para saturar reservas más rápido.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aumentá la fuerza máxima, la potencia explosiva y la masa muscular magra. La creatina es el suplemento más estudiado de la nutrición deportiva, con evidencia sólida para musculación, CrossFit, sprint y actividades de alta intensidad.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">creatina-star-300g-tabla.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">whey-gentech-500g-chocolate, combo-proteina-creatina-gentech</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://wa.me/5491124602875?text=Hola%2C%20me%20interesa%20la%20Creatina%20Monohidrato%20300g%20Star%20Nutrition</t>
-  </si>
-  <si>
-    <t xml:space="preserve">creatina-granger-300g</t>
-  </si>
-  <si>
     <t xml:space="preserve">Granger</t>
   </si>
   <si>
@@ -445,7 +448,13 @@
     <t xml:space="preserve">Maní</t>
   </si>
   <si>
+    <t xml:space="preserve">10 barras</t>
+  </si>
+  <si>
     <t xml:space="preserve">barrita-integra-mani-tabla.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">barrita-pont,</t>
   </si>
   <si>
     <t xml:space="preserve">https://wa.me/5491124602875?text=Hola%2C%20me%20interesa%20la%20Barrita%20Integra%20Man%C3%AD</t>
@@ -1188,7 +1197,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AB28"/>
-  <sheetFormatPr defaultColWidth="8.4921875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.4765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="35.84"/>
@@ -1197,11 +1206,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="38.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="14.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="14.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="14.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="14.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="17.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="16.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="10.83"/>
@@ -1211,11 +1220,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="18.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="10.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="28.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="23" style="0" width="90.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="23" style="0" width="90.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="38.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="55.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="90.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="50.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="90.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="50.82"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1345,7 +1354,7 @@
         <v>36</v>
       </c>
       <c r="I5" s="0" t="n">
-        <v>676767</v>
+        <v>666</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>37</v>
@@ -1413,10 +1422,10 @@
         <v>32</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G6" s="0" t="s">
         <v>35</v>
@@ -1428,16 +1437,16 @@
         <v>28000</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K6" s="0" t="s">
         <v>38</v>
       </c>
       <c r="O6" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R6" s="0" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="S6" s="0" t="s">
         <v>41</v>
@@ -1452,19 +1461,19 @@
         <v>44</v>
       </c>
       <c r="W6" s="0" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="X6" s="0" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="Y6" s="0" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Z6" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="AA6" s="0" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1472,7 +1481,7 @@
         <v>17</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C7" s="0" t="s">
         <v>32</v>
@@ -1481,10 +1490,10 @@
         <v>32</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G7" s="0" t="s">
         <v>35</v>
@@ -1496,40 +1505,40 @@
         <v>25500</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="O7" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R7" s="0" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="S7" s="0" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="T7" s="0" t="s">
         <v>42</v>
       </c>
       <c r="U7" s="0" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="V7" s="0" t="s">
         <v>44</v>
       </c>
       <c r="W7" s="0" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="X7" s="0" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Y7" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Z7" s="0" t="s">
         <v>48</v>
       </c>
       <c r="AA7" s="0" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1537,7 +1546,7 @@
         <v>1</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C8" s="0" t="s">
         <v>32</v>
@@ -1546,22 +1555,22 @@
         <v>32</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G8" s="0" t="s">
         <v>35</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I8" s="0" t="n">
         <v>34000</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="M8" s="0" t="s">
         <v>32</v>
@@ -1570,40 +1579,40 @@
         <v>2</v>
       </c>
       <c r="O8" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="P8" s="0" t="s">
         <v>32</v>
       </c>
       <c r="R8" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="S8" s="0" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="T8" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="U8" s="0" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="V8" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="W8" s="0" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="X8" s="0" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="Y8" s="0" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Z8" s="0" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="AA8" s="0" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1611,7 +1620,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C9" s="0" t="s">
         <v>32</v>
@@ -1620,55 +1629,55 @@
         <v>32</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G9" s="0" t="s">
         <v>35</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I9" s="0" t="n">
         <v>45000</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="O9" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R9" s="0" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="S9" s="0" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="T9" s="0" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="U9" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="V9" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="W9" s="0" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="X9" s="0" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="Y9" s="0" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="Z9" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="AA9" s="0" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1676,7 +1685,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C10" s="0" t="s">
         <v>32</v>
@@ -1685,22 +1694,22 @@
         <v>32</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G10" s="0" t="s">
         <v>35</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I10" s="0" t="n">
         <v>20000</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="M10" s="0" t="s">
         <v>32</v>
@@ -1709,34 +1718,34 @@
         <v>4</v>
       </c>
       <c r="O10" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R10" s="0" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="S10" s="0" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="T10" s="0" t="s">
         <v>42</v>
       </c>
       <c r="U10" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="V10" s="0" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="W10" s="0" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="X10" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="Y10" s="0" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AA10" s="0" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1744,7 +1753,7 @@
         <v>4</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C11" s="0" t="s">
         <v>32</v>
@@ -1753,52 +1762,52 @@
         <v>32</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G11" s="0" t="s">
         <v>35</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I11" s="0" t="n">
         <v>12000</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="O11" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R11" s="0" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="S11" s="0" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="T11" s="0" t="s">
         <v>42</v>
       </c>
       <c r="U11" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="V11" s="0" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="W11" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="X11" s="0" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="Y11" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AA11" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1806,7 +1815,7 @@
         <v>5</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C12" s="0" t="s">
         <v>32</v>
@@ -1815,55 +1824,55 @@
         <v>32</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I12" s="0" t="n">
         <v>20000</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K12" s="0" t="s">
         <v>38</v>
       </c>
       <c r="O12" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R12" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="S12" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="T12" s="0" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="U12" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="V12" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="W12" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="X12" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="Y12" s="0" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="AA12" s="0" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1871,7 +1880,7 @@
         <v>6</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C13" s="0" t="s">
         <v>32</v>
@@ -1880,55 +1889,58 @@
         <v>32</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I13" s="0" t="n">
         <v>20000</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="K13" s="0" t="s">
         <v>38</v>
       </c>
       <c r="O13" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R13" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="S13" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="T13" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="U13" s="0" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="V13" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="W13" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="X13" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="Y13" s="0" t="s">
-        <v>140</v>
+        <v>142</v>
+      </c>
+      <c r="Z13" s="0" t="s">
+        <v>143</v>
       </c>
       <c r="AA13" s="0" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1936,7 +1948,7 @@
         <v>7</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C14" s="0" t="s">
         <v>32</v>
@@ -1945,52 +1957,52 @@
         <v>32</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I14" s="0" t="n">
         <v>20000</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="O14" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R14" s="0" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="S14" s="0" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="T14" s="0" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="U14" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="V14" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="W14" s="0" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="X14" s="0" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="Y14" s="0" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="AA14" s="0" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1998,61 +2010,61 @@
         <v>8</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="C15" s="0" t="s">
         <v>32</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I15" s="0" t="n">
         <v>20000</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="O15" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R15" s="0" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="S15" s="0" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="T15" s="0" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="U15" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="V15" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="W15" s="0" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="X15" s="0" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="Y15" s="0" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="AA15" s="0" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2060,7 +2072,7 @@
         <v>9</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="C16" s="0" t="s">
         <v>32</v>
@@ -2069,55 +2081,55 @@
         <v>32</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I16" s="0" t="n">
         <v>20000</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="K16" s="0" t="s">
         <v>38</v>
       </c>
       <c r="O16" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R16" s="0" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="S16" s="0" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="T16" s="0" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="U16" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="V16" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="W16" s="0" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="X16" s="0" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="Y16" s="0" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="AA16" s="0" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2125,7 +2137,7 @@
         <v>10</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C17" s="0" t="s">
         <v>32</v>
@@ -2134,52 +2146,52 @@
         <v>32</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I17" s="0" t="n">
         <v>20000</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="O17" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R17" s="0" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="S17" s="0" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="T17" s="0" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U17" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="V17" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="W17" s="0" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="X17" s="0" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="Y17" s="0" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="AA17" s="0" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2187,7 +2199,7 @@
         <v>11</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C18" s="0" t="s">
         <v>32</v>
@@ -2196,52 +2208,52 @@
         <v>32</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I18" s="0" t="n">
         <v>20000</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="O18" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R18" s="0" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="S18" s="0" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="T18" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="U18" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="V18" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="W18" s="0" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="X18" s="0" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="Y18" s="0" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="AA18" s="0" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2249,7 +2261,7 @@
         <v>12</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="C19" s="0" t="s">
         <v>32</v>
@@ -2258,52 +2270,52 @@
         <v>32</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H19" s="0" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I19" s="0" t="n">
         <v>20000</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="O19" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R19" s="0" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="S19" s="0" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="T19" s="0" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="U19" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="V19" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="W19" s="0" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="X19" s="0" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="Y19" s="0" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="AA19" s="0" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2311,7 +2323,7 @@
         <v>13</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C20" s="0" t="s">
         <v>32</v>
@@ -2320,22 +2332,22 @@
         <v>32</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="G20" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H20" s="0" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="I20" s="0" t="n">
         <v>26500</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="M20" s="0" t="s">
         <v>32</v>
@@ -2344,40 +2356,40 @@
         <v>3</v>
       </c>
       <c r="O20" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="P20" s="0" t="s">
         <v>32</v>
       </c>
       <c r="R20" s="0" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="S20" s="0" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="T20" s="0" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="U20" s="0" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="V20" s="0" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="W20" s="0" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="X20" s="0" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="Y20" s="0" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="Z20" s="0" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="AA20" s="0" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2385,7 +2397,7 @@
         <v>18</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C21" s="0" t="s">
         <v>32</v>
@@ -2394,49 +2406,49 @@
         <v>32</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G21" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="H21" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="I21" s="0" t="n">
         <v>42000</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="O21" s="0" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="R21" s="0" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="S21" s="0" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="T21" s="0" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="U21" s="0" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="V21" s="0" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="W21" s="0" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="X21" s="0" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="AA21" s="0" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2444,7 +2456,7 @@
         <v>19</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="C22" s="0" t="s">
         <v>32</v>
@@ -2453,49 +2465,49 @@
         <v>32</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G22" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="H22" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="I22" s="0" t="n">
         <v>42000</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="O22" s="0" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="R22" s="0" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="S22" s="0" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="T22" s="0" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="U22" s="0" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="V22" s="0" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="W22" s="0" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="X22" s="0" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="AA22" s="0" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2503,7 +2515,7 @@
         <v>20</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C23" s="0" t="s">
         <v>32</v>
@@ -2512,49 +2524,49 @@
         <v>32</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="I23" s="0" t="n">
         <v>56000</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="O23" s="0" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="R23" s="0" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="S23" s="0" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="T23" s="0" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="U23" s="0" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="V23" s="0" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="W23" s="0" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="X23" s="0" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="AA23" s="0" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2562,7 +2574,7 @@
         <v>21</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="C24" s="0" t="s">
         <v>32</v>
@@ -2571,49 +2583,49 @@
         <v>32</v>
       </c>
       <c r="E24" s="0" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="I24" s="0" t="n">
         <v>90000</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="O24" s="0" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="R24" s="0" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="S24" s="0" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="T24" s="0" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="U24" s="0" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="V24" s="0" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="W24" s="0" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="X24" s="0" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="AA24" s="0" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2621,7 +2633,7 @@
         <v>22</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="C25" s="0" t="s">
         <v>32</v>
@@ -2630,22 +2642,22 @@
         <v>32</v>
       </c>
       <c r="E25" s="0" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="O25" s="0" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="P25" s="0" t="s">
         <v>32</v>
@@ -2654,31 +2666,31 @@
         <v>32</v>
       </c>
       <c r="R25" s="0" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="S25" s="0" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="T25" s="0" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="U25" s="0" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="V25" s="0" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="W25" s="0" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="X25" s="0" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="Z25" s="0" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="AA25" s="0" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2686,7 +2698,7 @@
         <v>23</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C26" s="0" t="s">
         <v>32</v>
@@ -2695,49 +2707,49 @@
         <v>32</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G26" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="H26" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="I26" s="0" t="n">
         <v>40000</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="O26" s="0" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="R26" s="0" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="S26" s="0" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="T26" s="0" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="U26" s="0" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="V26" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="W26" s="0" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="X26" s="0" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="AA26" s="0" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2745,7 +2757,7 @@
         <v>24</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="C27" s="0" t="s">
         <v>32</v>
@@ -2754,49 +2766,49 @@
         <v>32</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="H27" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="I27" s="0" t="n">
         <v>50000</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="O27" s="0" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="R27" s="0" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="S27" s="0" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="T27" s="0" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="U27" s="0" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="V27" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="W27" s="0" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="X27" s="0" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="AA27" s="0" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2804,31 +2816,31 @@
         <v>14</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D28" s="0" t="s">
         <v>32</v>
       </c>
       <c r="E28" s="0" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="H28" s="0" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="I28" s="0" t="n">
         <v>7400</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="K28" s="0" t="s">
         <v>38</v>
@@ -2840,37 +2852,37 @@
         <v>5</v>
       </c>
       <c r="O28" s="0" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="R28" s="0" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="S28" s="0" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="T28" s="0" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="U28" s="0" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="V28" s="0" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="W28" s="0" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="X28" s="0" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="Y28" s="0" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="Z28" s="0" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="AA28" s="0" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
     </row>
   </sheetData>
@@ -2890,98 +2902,98 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultColWidth="8.4921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.4765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="90.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="90.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="55.83"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2989,21 +3001,21 @@
         <v>30</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
     </row>
   </sheetData>
@@ -3023,179 +3035,179 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:A41"/>
-  <sheetFormatPr defaultColWidth="8.4921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.4765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="100.83"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
     </row>
   </sheetData>
@@ -3215,7 +3227,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="8.4921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.4765625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="2.83"/>
@@ -3223,12 +3235,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="2.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="2.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="50.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="50.82"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3242,7 +3254,7 @@
         <v>13</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3261,66 +3273,66 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C8" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C9" s="0" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C10" s="0" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C11" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C12" s="0" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizo catálogo y páginas de productos
</commit_message>
<xml_diff>
--- a/catalogo_productos_banco.xlsx
+++ b/catalogo_productos_banco.xlsx
@@ -1229,7 +1229,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AB30"/>
+  <dimension ref="A1:AB29"/>
   <sheetFormatPr defaultColWidth="10.4921875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.83"/>
@@ -2981,11 +2981,6 @@
         <v>296</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="n">
-        <v>26</v>
-      </c>
-    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511805555555555" footer="0.511805555555555"/>

</xml_diff>